<commit_message>
change the config dropdown to an options group inside a popover
</commit_message>
<xml_diff>
--- a/app/docs/Spreadhsheets/Scope Structure.xlsx
+++ b/app/docs/Spreadhsheets/Scope Structure.xlsx
@@ -5,15 +5,16 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/robhay/Developer/share_screener/app/docs/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/robhay/Developer/share_screener/app/docs/Spreadhsheets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{093CDC4D-17CA-FA45-8391-C320CD0A9D89}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5ABD55C9-F674-F045-AEC4-664C7DBDDE3D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="21580" xr2:uid="{952C95C7-3405-C54E-B78D-3397068AE8B3}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="21580" activeTab="1" xr2:uid="{952C95C7-3405-C54E-B78D-3397068AE8B3}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1 (2)" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="329" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="503" uniqueCount="120">
   <si>
     <t>Scope</t>
   </si>
@@ -337,13 +338,67 @@
   </si>
   <si>
     <t>show_config_verdicts</t>
+  </si>
+  <si>
+    <t>Names</t>
+  </si>
+  <si>
+    <t>Module</t>
+  </si>
+  <si>
+    <t>Function</t>
+  </si>
+  <si>
+    <t>Config
+(View)</t>
+  </si>
+  <si>
+    <t>Scope
+(Create)</t>
+  </si>
+  <si>
+    <t>Page</t>
+  </si>
+  <si>
+    <t>Settings
+Button</t>
+  </si>
+  <si>
+    <t>Dropdown
+List</t>
+  </si>
+  <si>
+    <t>Config
+Button</t>
+  </si>
+  <si>
+    <t>Page(s)
+ access to the above code</t>
+  </si>
+  <si>
+    <t>Config Groups</t>
+  </si>
+  <si>
+    <t>Path</t>
+  </si>
+  <si>
+    <t>Syntax</t>
+  </si>
+  <si>
+    <t>Notes</t>
+  </si>
+  <si>
+    <t>Altenative Name</t>
+  </si>
+  <si>
+    <t>overview of all scope</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="17" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -477,6 +532,22 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <i/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FF00B0F0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="8">
     <fill>
@@ -522,7 +593,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="8">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -619,11 +690,40 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="60">
+  <cellXfs count="93">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -656,9 +756,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -668,14 +765,8 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -708,95 +799,203 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1127,12 +1326,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:25" ht="26" x14ac:dyDescent="0.3">
-      <c r="A1" s="19" t="s">
+      <c r="A1" s="16" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="2" spans="1:25" x14ac:dyDescent="0.2">
-      <c r="H2" s="45" t="s">
+      <c r="H2" s="33" t="s">
         <v>59</v>
       </c>
       <c r="J2" s="4" t="s">
@@ -1140,172 +1339,172 @@
       </c>
     </row>
     <row r="5" spans="1:25" ht="26" x14ac:dyDescent="0.2">
-      <c r="C5" s="18" t="s">
+      <c r="C5" s="58" t="s">
         <v>37</v>
       </c>
-      <c r="D5" s="37" t="s">
+      <c r="D5" s="47" t="s">
         <v>31</v>
       </c>
-      <c r="E5" s="37" t="s">
+      <c r="E5" s="47" t="s">
         <v>1</v>
       </c>
-      <c r="F5" s="37" t="s">
+      <c r="F5" s="47" t="s">
         <v>99</v>
       </c>
-      <c r="H5" s="40" t="s">
+      <c r="H5" s="56" t="s">
         <v>0</v>
       </c>
-      <c r="I5" s="40"/>
-      <c r="J5" s="33" t="s">
+      <c r="I5" s="56"/>
+      <c r="J5" s="53" t="s">
         <v>74</v>
       </c>
-      <c r="K5" s="33"/>
-      <c r="L5" s="33" t="s">
+      <c r="K5" s="53"/>
+      <c r="L5" s="53" t="s">
         <v>75</v>
       </c>
-      <c r="M5" s="33"/>
-      <c r="N5" s="16" t="s">
+      <c r="M5" s="53"/>
+      <c r="N5" s="42" t="s">
         <v>84</v>
       </c>
-      <c r="O5" s="16"/>
-      <c r="P5" s="16"/>
-      <c r="Q5" s="16"/>
-      <c r="R5" s="16"/>
-      <c r="S5" s="16"/>
-      <c r="T5" s="16"/>
-      <c r="U5" s="16"/>
-      <c r="V5" s="16"/>
-      <c r="W5" s="16"/>
-      <c r="X5" s="16"/>
-      <c r="Y5" s="16"/>
-    </row>
-    <row r="6" spans="1:25" s="15" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C6" s="18"/>
-      <c r="D6" s="38"/>
-      <c r="E6" s="38"/>
-      <c r="F6" s="38"/>
-      <c r="G6" s="21"/>
-      <c r="H6" s="36" t="s">
+      <c r="O5" s="42"/>
+      <c r="P5" s="42"/>
+      <c r="Q5" s="42"/>
+      <c r="R5" s="42"/>
+      <c r="S5" s="42"/>
+      <c r="T5" s="42"/>
+      <c r="U5" s="42"/>
+      <c r="V5" s="42"/>
+      <c r="W5" s="42"/>
+      <c r="X5" s="42"/>
+      <c r="Y5" s="42"/>
+    </row>
+    <row r="6" spans="1:25" s="14" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C6" s="58"/>
+      <c r="D6" s="48"/>
+      <c r="E6" s="48"/>
+      <c r="F6" s="48"/>
+      <c r="G6" s="18"/>
+      <c r="H6" s="59" t="s">
         <v>79</v>
       </c>
-      <c r="I6" s="36"/>
-      <c r="J6" s="43" t="s">
+      <c r="I6" s="59"/>
+      <c r="J6" s="54" t="s">
         <v>80</v>
       </c>
-      <c r="K6" s="44"/>
-      <c r="L6" s="43" t="s">
+      <c r="K6" s="55"/>
+      <c r="L6" s="54" t="s">
         <v>81</v>
       </c>
-      <c r="M6" s="44"/>
-      <c r="N6" s="17" t="s">
+      <c r="M6" s="55"/>
+      <c r="N6" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="O6" s="17" t="s">
+      <c r="O6" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="P6" s="50" t="s">
+      <c r="P6" s="36" t="s">
         <v>20</v>
       </c>
-      <c r="Q6" s="17" t="s">
+      <c r="Q6" s="15" t="s">
         <v>96</v>
       </c>
-      <c r="R6" s="17" t="s">
+      <c r="R6" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="S6" s="17" t="s">
+      <c r="S6" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="T6" s="17" t="s">
+      <c r="T6" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="U6" s="17" t="s">
+      <c r="U6" s="15" t="s">
         <v>29</v>
       </c>
-      <c r="V6" s="17" t="s">
+      <c r="V6" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="W6" s="17" t="s">
+      <c r="W6" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="X6" s="26" t="s">
+      <c r="X6" s="23" t="s">
         <v>19</v>
       </c>
-      <c r="Y6" s="26" t="s">
+      <c r="Y6" s="23" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="7" spans="1:25" s="15" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C7" s="20"/>
-      <c r="D7" s="20"/>
-      <c r="E7" s="20"/>
-      <c r="F7" s="20"/>
-      <c r="G7" s="21"/>
-      <c r="H7" s="41" t="s">
+    <row r="7" spans="1:25" s="14" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C7" s="17"/>
+      <c r="D7" s="17"/>
+      <c r="E7" s="17"/>
+      <c r="F7" s="17"/>
+      <c r="G7" s="18"/>
+      <c r="H7" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="I7" s="41" t="s">
+      <c r="I7" s="31" t="s">
         <v>48</v>
       </c>
-      <c r="J7" s="41" t="s">
+      <c r="J7" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="K7" s="41" t="s">
+      <c r="K7" s="31" t="s">
         <v>48</v>
       </c>
-      <c r="L7" s="39"/>
-      <c r="M7" s="39"/>
-      <c r="N7" s="28" t="s">
+      <c r="L7" s="30"/>
+      <c r="M7" s="30"/>
+      <c r="N7" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="O7" s="28" t="s">
+      <c r="O7" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="P7" s="28" t="s">
+      <c r="P7" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="Q7" s="28" t="s">
+      <c r="Q7" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="R7" s="28" t="s">
+      <c r="R7" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="S7" s="28" t="s">
+      <c r="S7" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="T7" s="28" t="s">
+      <c r="T7" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="U7" s="28" t="s">
+      <c r="U7" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="V7" s="28" t="s">
+      <c r="V7" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="W7" s="28" t="s">
+      <c r="W7" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="X7" s="26" t="s">
+      <c r="X7" s="23" t="s">
         <v>18</v>
       </c>
-      <c r="Y7" s="26" t="s">
+      <c r="Y7" s="23" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="8" spans="1:25" s="8" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C8" s="15" t="s">
+      <c r="C8" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="G8" s="21"/>
-      <c r="H8" s="42" t="s">
+      <c r="G8" s="18"/>
+      <c r="H8" s="32" t="s">
         <v>47</v>
       </c>
-      <c r="I8" s="42" t="s">
+      <c r="I8" s="32" t="s">
         <v>47</v>
       </c>
-      <c r="J8" s="27" t="s">
+      <c r="J8" s="24" t="s">
         <v>13</v>
       </c>
-      <c r="K8" s="27" t="s">
+      <c r="K8" s="24" t="s">
         <v>14</v>
       </c>
       <c r="L8" s="7" t="s">
@@ -1316,12 +1515,12 @@
       </c>
     </row>
     <row r="9" spans="1:25" s="8" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C9" s="20"/>
-      <c r="D9" s="20"/>
-      <c r="G9" s="21"/>
-      <c r="H9" s="21"/>
-      <c r="I9" s="21"/>
-      <c r="K9" s="56" t="s">
+      <c r="C9" s="17"/>
+      <c r="D9" s="17"/>
+      <c r="G9" s="18"/>
+      <c r="H9" s="18"/>
+      <c r="I9" s="18"/>
+      <c r="K9" s="40" t="s">
         <v>85</v>
       </c>
     </row>
@@ -1342,196 +1541,196 @@
       </c>
       <c r="F11" s="6"/>
       <c r="G11" s="6"/>
-      <c r="H11" s="25" t="s">
+      <c r="H11" s="22" t="s">
         <v>58</v>
       </c>
-      <c r="I11" s="25" t="s">
+      <c r="I11" s="22" t="s">
         <v>58</v>
       </c>
-      <c r="J11" s="46" t="s">
+      <c r="J11" s="34" t="s">
         <v>69</v>
       </c>
-      <c r="K11" s="46" t="s">
+      <c r="K11" s="34" t="s">
         <v>87</v>
       </c>
-      <c r="L11" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="M11" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="N11" s="51" t="s">
+      <c r="L11" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="M11" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="N11" s="37" t="s">
         <v>45</v>
       </c>
-      <c r="O11" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="P11" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q11" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="R11" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="S11" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="T11" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="U11" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="V11" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="W11" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="X11" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y11" s="25" t="s">
+      <c r="O11" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="P11" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q11" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="R11" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="S11" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="T11" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="U11" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="V11" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="W11" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="X11" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y11" s="22" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="12" spans="1:25" s="10" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="C12" s="23" t="s">
+      <c r="C12" s="20" t="s">
         <v>3</v>
       </c>
-      <c r="D12" s="12" t="s">
+      <c r="D12" s="11" t="s">
         <v>34</v>
       </c>
       <c r="E12" s="9"/>
       <c r="F12" s="9"/>
       <c r="G12" s="9"/>
-      <c r="H12" s="46" t="s">
+      <c r="H12" s="34" t="s">
         <v>51</v>
       </c>
-      <c r="I12" s="46" t="s">
+      <c r="I12" s="34" t="s">
         <v>51</v>
       </c>
-      <c r="J12" s="46" t="s">
+      <c r="J12" s="34" t="s">
         <v>68</v>
       </c>
-      <c r="K12" s="46" t="s">
+      <c r="K12" s="34" t="s">
         <v>86</v>
       </c>
-      <c r="L12" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="M12" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="N12" s="51" t="s">
+      <c r="L12" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="M12" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="N12" s="37" t="s">
         <v>45</v>
       </c>
-      <c r="O12" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="P12" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q12" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="R12" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="S12" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="T12" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="U12" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="V12" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="W12" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="X12" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y12" s="25" t="s">
+      <c r="O12" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="P12" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q12" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="R12" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="S12" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="T12" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="U12" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="V12" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="W12" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="X12" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y12" s="22" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="13" spans="1:25" s="10" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="C13" s="23" t="s">
+      <c r="C13" s="20" t="s">
         <v>4</v>
       </c>
-      <c r="D13" s="12" t="s">
+      <c r="D13" s="11" t="s">
         <v>34</v>
       </c>
       <c r="E13" s="9"/>
       <c r="F13" s="9"/>
       <c r="G13" s="9"/>
-      <c r="H13" s="46" t="s">
+      <c r="H13" s="34" t="s">
         <v>50</v>
       </c>
-      <c r="I13" s="46" t="s">
+      <c r="I13" s="34" t="s">
         <v>50</v>
       </c>
-      <c r="J13" s="46" t="s">
+      <c r="J13" s="34" t="s">
         <v>61</v>
       </c>
-      <c r="K13" s="46" t="s">
+      <c r="K13" s="34" t="s">
         <v>87</v>
       </c>
-      <c r="L13" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="M13" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="N13" s="51" t="s">
+      <c r="L13" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="M13" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="N13" s="37" t="s">
         <v>45</v>
       </c>
-      <c r="O13" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="P13" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q13" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="R13" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="S13" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="T13" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="U13" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="V13" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="W13" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="X13" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y13" s="25" t="s">
+      <c r="O13" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="P13" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q13" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="R13" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="S13" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="T13" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="U13" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="V13" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="W13" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="X13" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y13" s="22" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="14" spans="1:25" s="10" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="C14" s="23" t="s">
+      <c r="C14" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="D14" s="14" t="s">
+      <c r="D14" s="13" t="s">
         <v>32</v>
       </c>
       <c r="E14" s="9"/>
@@ -1539,134 +1738,134 @@
         <v>100</v>
       </c>
       <c r="G14" s="9"/>
-      <c r="H14" s="46" t="s">
+      <c r="H14" s="34" t="s">
         <v>49</v>
       </c>
-      <c r="I14" s="46" t="s">
+      <c r="I14" s="34" t="s">
         <v>49</v>
       </c>
-      <c r="J14" s="46" t="s">
+      <c r="J14" s="34" t="s">
         <v>67</v>
       </c>
-      <c r="K14" s="46" t="s">
+      <c r="K14" s="34" t="s">
         <v>88</v>
       </c>
-      <c r="L14" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="M14" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="N14" s="51" t="s">
+      <c r="L14" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="M14" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="N14" s="37" t="s">
         <v>45</v>
       </c>
-      <c r="O14" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="P14" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q14" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="R14" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="S14" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="T14" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="U14" s="54" t="s">
+      <c r="O14" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="P14" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q14" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="R14" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="S14" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="T14" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="U14" s="38" t="s">
         <v>101</v>
       </c>
-      <c r="V14" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="W14" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="X14" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y14" s="25" t="s">
+      <c r="V14" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="W14" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="X14" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y14" s="22" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="15" spans="1:25" s="10" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="C15" s="23" t="s">
+      <c r="C15" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="D15" s="12" t="s">
+      <c r="D15" s="11" t="s">
         <v>34</v>
       </c>
       <c r="E15" s="9"/>
       <c r="F15" s="9"/>
       <c r="G15" s="9"/>
-      <c r="H15" s="47" t="s">
+      <c r="H15" s="35" t="s">
         <v>46</v>
       </c>
-      <c r="I15" s="47" t="s">
+      <c r="I15" s="35" t="s">
         <v>46</v>
       </c>
-      <c r="J15" s="46" t="s">
+      <c r="J15" s="34" t="s">
         <v>60</v>
       </c>
-      <c r="K15" s="46" t="s">
+      <c r="K15" s="34" t="s">
         <v>89</v>
       </c>
-      <c r="L15" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="M15" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="N15" s="51" t="s">
+      <c r="L15" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="M15" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="N15" s="37" t="s">
         <v>45</v>
       </c>
-      <c r="O15" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="P15" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q15" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="R15" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="S15" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="T15" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="U15" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="V15" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="W15" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="X15" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y15" s="25" t="s">
+      <c r="O15" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="P15" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q15" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="R15" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="S15" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="T15" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="U15" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="V15" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="W15" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="X15" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y15" s="22" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="16" spans="1:25" s="10" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="B16" s="11" t="s">
+      <c r="B16" s="57" t="s">
         <v>30</v>
       </c>
-      <c r="C16" s="57" t="s">
+      <c r="C16" s="45" t="s">
         <v>7</v>
       </c>
-      <c r="D16" s="14" t="s">
+      <c r="D16" s="13" t="s">
         <v>32</v>
       </c>
       <c r="E16" s="9" t="s">
@@ -1676,254 +1875,254 @@
         <v>100</v>
       </c>
       <c r="G16" s="9"/>
-      <c r="H16" s="48" t="s">
+      <c r="H16" s="49" t="s">
         <v>52</v>
       </c>
-      <c r="I16" s="48" t="s">
+      <c r="I16" s="49" t="s">
         <v>52</v>
       </c>
-      <c r="J16" s="46" t="s">
+      <c r="J16" s="34" t="s">
         <v>64</v>
       </c>
-      <c r="K16" s="46" t="s">
+      <c r="K16" s="34" t="s">
         <v>90</v>
       </c>
-      <c r="L16" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="M16" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="N16" s="51" t="s">
+      <c r="L16" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="M16" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="N16" s="37" t="s">
         <v>45</v>
       </c>
-      <c r="O16" s="59" t="s">
+      <c r="O16" s="41" t="s">
         <v>101</v>
       </c>
-      <c r="P16" s="54" t="s">
+      <c r="P16" s="38" t="s">
         <v>101</v>
       </c>
-      <c r="Q16" s="54" t="s">
+      <c r="Q16" s="38" t="s">
         <v>101</v>
       </c>
-      <c r="R16" s="54" t="s">
+      <c r="R16" s="38" t="s">
         <v>101</v>
       </c>
-      <c r="S16" s="25" t="s">
+      <c r="S16" s="22" t="s">
         <v>58</v>
       </c>
-      <c r="T16" s="25" t="s">
+      <c r="T16" s="22" t="s">
         <v>58</v>
       </c>
-      <c r="U16" s="25" t="s">
+      <c r="U16" s="22" t="s">
         <v>58</v>
       </c>
-      <c r="V16" s="25" t="s">
+      <c r="V16" s="22" t="s">
         <v>58</v>
       </c>
-      <c r="W16" s="54" t="s">
+      <c r="W16" s="38" t="s">
         <v>101</v>
       </c>
-      <c r="X16" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y16" s="25" t="s">
+      <c r="X16" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y16" s="22" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="17" spans="2:25" s="10" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B17" s="11"/>
-      <c r="C17" s="58"/>
-      <c r="D17" s="29" t="s">
+      <c r="B17" s="57"/>
+      <c r="C17" s="46"/>
+      <c r="D17" s="26" t="s">
         <v>98</v>
       </c>
       <c r="E17" s="9"/>
       <c r="F17" s="9"/>
       <c r="G17" s="9"/>
-      <c r="H17" s="49"/>
-      <c r="I17" s="49"/>
-      <c r="J17" s="46" t="s">
+      <c r="H17" s="50"/>
+      <c r="I17" s="50"/>
+      <c r="J17" s="34" t="s">
         <v>102</v>
       </c>
-      <c r="K17" s="46" t="s">
+      <c r="K17" s="34" t="s">
         <v>103</v>
       </c>
-      <c r="L17" s="25"/>
-      <c r="M17" s="25"/>
-      <c r="N17" s="51" t="s">
+      <c r="L17" s="22"/>
+      <c r="M17" s="22"/>
+      <c r="N17" s="37" t="s">
         <v>45</v>
       </c>
-      <c r="O17" s="54" t="s">
+      <c r="O17" s="38" t="s">
         <v>101</v>
       </c>
-      <c r="P17" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q17" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="R17" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="S17" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="T17" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="U17" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="V17" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="W17" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="X17" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y17" s="25" t="s">
+      <c r="P17" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q17" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="R17" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="S17" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="T17" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="U17" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="V17" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="W17" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="X17" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y17" s="22" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="18" spans="2:25" s="10" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="B18" s="11"/>
-      <c r="C18" s="23" t="s">
+      <c r="B18" s="57"/>
+      <c r="C18" s="20" t="s">
         <v>8</v>
       </c>
-      <c r="D18" s="12" t="s">
+      <c r="D18" s="11" t="s">
         <v>34</v>
       </c>
       <c r="E18" s="9"/>
       <c r="F18" s="9"/>
       <c r="G18" s="9"/>
-      <c r="H18" s="46" t="s">
+      <c r="H18" s="34" t="s">
         <v>53</v>
       </c>
-      <c r="I18" s="46" t="s">
+      <c r="I18" s="34" t="s">
         <v>53</v>
       </c>
-      <c r="J18" s="46" t="s">
+      <c r="J18" s="34" t="s">
         <v>66</v>
       </c>
-      <c r="K18" s="46" t="s">
+      <c r="K18" s="34" t="s">
         <v>91</v>
       </c>
-      <c r="L18" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="M18" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="N18" s="51" t="s">
+      <c r="L18" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="M18" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="N18" s="37" t="s">
         <v>45</v>
       </c>
-      <c r="O18" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="P18" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q18" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="R18" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="S18" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="T18" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="U18" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="V18" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="W18" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="X18" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y18" s="25" t="s">
+      <c r="O18" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="P18" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q18" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="R18" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="S18" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="T18" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="U18" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="V18" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="W18" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="X18" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y18" s="22" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="19" spans="2:25" s="10" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="B19" s="11"/>
-      <c r="C19" s="23" t="s">
+      <c r="B19" s="57"/>
+      <c r="C19" s="20" t="s">
         <v>9</v>
       </c>
-      <c r="D19" s="12" t="s">
+      <c r="D19" s="11" t="s">
         <v>34</v>
       </c>
       <c r="E19" s="9"/>
       <c r="F19" s="9"/>
       <c r="G19" s="9"/>
-      <c r="H19" s="46" t="s">
+      <c r="H19" s="34" t="s">
         <v>63</v>
       </c>
-      <c r="I19" s="46" t="s">
+      <c r="I19" s="34" t="s">
         <v>63</v>
       </c>
-      <c r="J19" s="46" t="s">
+      <c r="J19" s="34" t="s">
         <v>65</v>
       </c>
-      <c r="K19" s="46" t="s">
+      <c r="K19" s="34" t="s">
         <v>92</v>
       </c>
-      <c r="L19" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="M19" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="N19" s="51" t="s">
+      <c r="L19" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="M19" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="N19" s="37" t="s">
         <v>45</v>
       </c>
-      <c r="O19" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="P19" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q19" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="R19" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="S19" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="T19" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="U19" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="V19" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="W19" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="X19" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y19" s="25" t="s">
+      <c r="O19" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="P19" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q19" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="R19" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="S19" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="T19" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="U19" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="V19" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="W19" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="X19" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y19" s="22" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="20" spans="2:25" s="10" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="C20" s="23" t="s">
+      <c r="C20" s="20" t="s">
         <v>10</v>
       </c>
-      <c r="D20" s="12" t="s">
+      <c r="D20" s="11" t="s">
         <v>34</v>
       </c>
       <c r="E20" s="9"/>
@@ -1931,69 +2130,69 @@
         <v>100</v>
       </c>
       <c r="G20" s="9"/>
-      <c r="H20" s="46" t="s">
+      <c r="H20" s="34" t="s">
         <v>54</v>
       </c>
-      <c r="I20" s="46" t="s">
+      <c r="I20" s="34" t="s">
         <v>54</v>
       </c>
-      <c r="J20" s="46" t="s">
+      <c r="J20" s="34" t="s">
         <v>62</v>
       </c>
-      <c r="K20" s="46" t="s">
+      <c r="K20" s="34" t="s">
         <v>97</v>
       </c>
-      <c r="L20" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="M20" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="N20" s="51" t="s">
+      <c r="L20" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="M20" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="N20" s="37" t="s">
         <v>45</v>
       </c>
-      <c r="O20" s="54" t="s">
+      <c r="O20" s="38" t="s">
         <v>101</v>
       </c>
-      <c r="P20" s="54" t="s">
+      <c r="P20" s="38" t="s">
         <v>101</v>
       </c>
-      <c r="Q20" s="54" t="s">
+      <c r="Q20" s="38" t="s">
         <v>101</v>
       </c>
-      <c r="R20" s="54" t="s">
+      <c r="R20" s="38" t="s">
         <v>101</v>
       </c>
-      <c r="S20" s="54" t="s">
+      <c r="S20" s="38" t="s">
         <v>101</v>
       </c>
-      <c r="T20" s="54" t="s">
+      <c r="T20" s="38" t="s">
         <v>101</v>
       </c>
-      <c r="U20" s="54" t="s">
+      <c r="U20" s="38" t="s">
         <v>101</v>
       </c>
-      <c r="V20" s="25" t="s">
+      <c r="V20" s="22" t="s">
         <v>58</v>
       </c>
-      <c r="W20" s="25" t="s">
+      <c r="W20" s="22" t="s">
         <v>58</v>
       </c>
-      <c r="X20" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y20" s="25" t="s">
+      <c r="X20" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y20" s="22" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="21" spans="2:25" s="10" customFormat="1" ht="34" x14ac:dyDescent="0.2">
-      <c r="B21" s="11" t="s">
+      <c r="B21" s="57" t="s">
         <v>19</v>
       </c>
-      <c r="C21" s="23" t="s">
+      <c r="C21" s="20" t="s">
         <v>39</v>
       </c>
-      <c r="D21" s="12" t="s">
+      <c r="D21" s="11" t="s">
         <v>34</v>
       </c>
       <c r="E21" s="9" t="s">
@@ -2001,267 +2200,275 @@
       </c>
       <c r="F21" s="9"/>
       <c r="G21" s="9"/>
-      <c r="H21" s="46" t="s">
+      <c r="H21" s="34" t="s">
         <v>55</v>
       </c>
-      <c r="I21" s="46" t="s">
+      <c r="I21" s="34" t="s">
         <v>55</v>
       </c>
-      <c r="J21" s="46" t="s">
+      <c r="J21" s="34" t="s">
         <v>71</v>
       </c>
-      <c r="K21" s="46" t="s">
+      <c r="K21" s="34" t="s">
         <v>93</v>
       </c>
-      <c r="L21" s="46" t="s">
+      <c r="L21" s="34" t="s">
         <v>82</v>
       </c>
-      <c r="M21" s="46" t="s">
+      <c r="M21" s="34" t="s">
         <v>83</v>
       </c>
-      <c r="N21" s="51" t="s">
+      <c r="N21" s="37" t="s">
         <v>45</v>
       </c>
-      <c r="O21" s="54" t="s">
+      <c r="O21" s="38" t="s">
         <v>101</v>
       </c>
-      <c r="P21" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q21" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="R21" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="S21" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="T21" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="U21" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="V21" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="W21" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="X21" s="55" t="s">
+      <c r="P21" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q21" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="R21" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="S21" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="T21" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="U21" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="V21" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="W21" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="X21" s="39" t="s">
         <v>43</v>
       </c>
-      <c r="Y21" s="25" t="s">
+      <c r="Y21" s="22" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="22" spans="2:25" s="10" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="B22" s="11"/>
-      <c r="C22" s="23" t="s">
+      <c r="B22" s="57"/>
+      <c r="C22" s="20" t="s">
         <v>11</v>
       </c>
-      <c r="D22" s="12" t="s">
+      <c r="D22" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="E22" s="24" t="s">
+      <c r="E22" s="21" t="s">
         <v>41</v>
       </c>
-      <c r="F22" s="24"/>
-      <c r="G22" s="24"/>
-      <c r="H22" s="46" t="s">
+      <c r="F22" s="21"/>
+      <c r="G22" s="21"/>
+      <c r="H22" s="34" t="s">
         <v>56</v>
       </c>
-      <c r="I22" s="46" t="s">
+      <c r="I22" s="34" t="s">
         <v>56</v>
       </c>
-      <c r="J22" s="46" t="s">
+      <c r="J22" s="34" t="s">
         <v>70</v>
       </c>
-      <c r="K22" s="46" t="s">
+      <c r="K22" s="34" t="s">
         <v>94</v>
       </c>
-      <c r="L22" s="32" t="s">
+      <c r="L22" s="27" t="s">
         <v>44</v>
       </c>
-      <c r="M22" s="32" t="s">
+      <c r="M22" s="27" t="s">
         <v>44</v>
       </c>
-      <c r="N22" s="51" t="s">
+      <c r="N22" s="37" t="s">
         <v>45</v>
       </c>
-      <c r="O22" s="54" t="s">
+      <c r="O22" s="38" t="s">
         <v>101</v>
       </c>
-      <c r="P22" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q22" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="R22" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="S22" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="T22" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="U22" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="V22" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="W22" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="X22" s="32" t="s">
+      <c r="P22" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q22" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="R22" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="S22" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="T22" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="U22" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="V22" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="W22" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="X22" s="27" t="s">
         <v>44</v>
       </c>
-      <c r="Y22" s="25" t="s">
+      <c r="Y22" s="22" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="23" spans="2:25" s="10" customFormat="1" ht="34" x14ac:dyDescent="0.2">
-      <c r="B23" s="11" t="s">
+      <c r="B23" s="57" t="s">
         <v>20</v>
       </c>
-      <c r="C23" s="23" t="s">
+      <c r="C23" s="20" t="s">
         <v>36</v>
       </c>
-      <c r="D23" s="12" t="s">
+      <c r="D23" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="E23" s="22"/>
-      <c r="F23" s="22"/>
-      <c r="G23" s="34"/>
-      <c r="H23" s="48" t="s">
+      <c r="E23" s="19"/>
+      <c r="F23" s="19"/>
+      <c r="G23" s="28"/>
+      <c r="H23" s="49" t="s">
         <v>57</v>
       </c>
-      <c r="I23" s="48" t="s">
+      <c r="I23" s="49" t="s">
         <v>57</v>
       </c>
-      <c r="J23" s="48" t="s">
+      <c r="J23" s="49" t="s">
         <v>72</v>
       </c>
-      <c r="K23" s="48" t="s">
+      <c r="K23" s="49" t="s">
         <v>95</v>
       </c>
-      <c r="L23" s="46" t="s">
+      <c r="L23" s="34" t="s">
         <v>73</v>
       </c>
-      <c r="M23" s="46" t="s">
+      <c r="M23" s="34" t="s">
         <v>76</v>
       </c>
-      <c r="N23" s="52" t="s">
+      <c r="N23" s="51" t="s">
         <v>45</v>
       </c>
-      <c r="O23" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="P23" s="30" t="s">
+      <c r="O23" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="P23" s="43" t="s">
         <v>101</v>
       </c>
-      <c r="Q23" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="R23" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="S23" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="T23" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="U23" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="V23" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="W23" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="X23" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y23" s="55" t="s">
+      <c r="Q23" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="R23" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="S23" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="T23" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="U23" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="V23" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="W23" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="X23" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y23" s="39" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="24" spans="2:25" ht="34" x14ac:dyDescent="0.2">
-      <c r="B24" s="11"/>
+      <c r="B24" s="57"/>
       <c r="C24" s="9"/>
-      <c r="D24" s="12" t="s">
+      <c r="D24" s="11" t="s">
         <v>34</v>
       </c>
       <c r="E24" s="9" t="s">
         <v>35</v>
       </c>
       <c r="F24" s="9"/>
-      <c r="G24" s="35"/>
-      <c r="H24" s="49"/>
-      <c r="I24" s="49"/>
-      <c r="J24" s="49"/>
-      <c r="K24" s="49"/>
-      <c r="L24" s="46" t="s">
+      <c r="G24" s="29"/>
+      <c r="H24" s="50"/>
+      <c r="I24" s="50"/>
+      <c r="J24" s="50"/>
+      <c r="K24" s="50"/>
+      <c r="L24" s="34" t="s">
         <v>77</v>
       </c>
-      <c r="M24" s="46" t="s">
+      <c r="M24" s="34" t="s">
         <v>78</v>
       </c>
-      <c r="N24" s="53"/>
-      <c r="O24" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="P24" s="31"/>
-      <c r="Q24" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="R24" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="S24" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="T24" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="U24" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="V24" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="W24" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="X24" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="Y24" s="55" t="s">
+      <c r="N24" s="52"/>
+      <c r="O24" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="P24" s="44"/>
+      <c r="Q24" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="R24" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="S24" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="T24" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="U24" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="V24" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="W24" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="X24" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y24" s="39" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="27" spans="2:25" ht="21" x14ac:dyDescent="0.25">
       <c r="C27" s="1"/>
-      <c r="D27" s="13"/>
+      <c r="D27" s="12"/>
     </row>
     <row r="28" spans="2:25" ht="21" x14ac:dyDescent="0.25">
       <c r="C28" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="D28" s="13"/>
+      <c r="D28" s="12"/>
     </row>
     <row r="29" spans="2:25" ht="21" x14ac:dyDescent="0.25">
       <c r="C29" s="1"/>
-      <c r="D29" s="13"/>
+      <c r="D29" s="12"/>
     </row>
   </sheetData>
   <mergeCells count="23">
+    <mergeCell ref="B21:B22"/>
+    <mergeCell ref="B23:B24"/>
+    <mergeCell ref="J23:J24"/>
+    <mergeCell ref="K23:K24"/>
+    <mergeCell ref="L6:M6"/>
+    <mergeCell ref="B16:B19"/>
+    <mergeCell ref="C5:C6"/>
+    <mergeCell ref="H6:I6"/>
     <mergeCell ref="N5:Y5"/>
     <mergeCell ref="P23:P24"/>
     <mergeCell ref="C16:C17"/>
@@ -2277,14 +2484,839 @@
     <mergeCell ref="H23:H24"/>
     <mergeCell ref="I23:I24"/>
     <mergeCell ref="L5:M5"/>
-    <mergeCell ref="B21:B22"/>
-    <mergeCell ref="B23:B24"/>
-    <mergeCell ref="J23:J24"/>
-    <mergeCell ref="K23:K24"/>
-    <mergeCell ref="L6:M6"/>
-    <mergeCell ref="B16:B19"/>
-    <mergeCell ref="C5:C6"/>
-    <mergeCell ref="H6:I6"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14994931-7C6C-9340-B5B5-F2DD8D95EA73}">
+  <dimension ref="A1:AF27"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="4.1640625" style="10" customWidth="1"/>
+    <col min="2" max="2" width="15.6640625" style="10" customWidth="1"/>
+    <col min="3" max="3" width="27.6640625" style="10" customWidth="1"/>
+    <col min="4" max="4" width="9.1640625" style="10" customWidth="1"/>
+    <col min="5" max="5" width="19.6640625" style="75" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="6" style="75" customWidth="1"/>
+    <col min="7" max="7" width="18.33203125" style="10" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="16" style="10" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="17.6640625" style="10" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="22.6640625" style="10" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="17" style="10" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="18" style="10" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="19" style="10" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="25.5" style="10" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="14" style="10" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="17.5" style="10" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="18.33203125" style="10" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="19.33203125" style="10" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="19.1640625" style="10" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="20" style="10" bestFit="1" customWidth="1"/>
+    <col min="21" max="16384" width="10.83203125" style="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:20" ht="26" x14ac:dyDescent="0.2">
+      <c r="A1" s="76" t="s">
+        <v>40</v>
+      </c>
+      <c r="B1" s="76"/>
+      <c r="C1" s="76"/>
+      <c r="D1" s="76"/>
+      <c r="E1" s="77"/>
+      <c r="F1" s="77"/>
+      <c r="G1" s="76"/>
+      <c r="H1" s="76"/>
+      <c r="I1" s="76"/>
+      <c r="J1" s="76"/>
+      <c r="S1" s="76"/>
+      <c r="T1" s="76"/>
+    </row>
+    <row r="3" spans="1:20" s="61" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="E3" s="89" t="s">
+        <v>114</v>
+      </c>
+      <c r="G3" s="22"/>
+      <c r="H3" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="I3" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="J3" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="K3" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="L3" s="83" t="s">
+        <v>7</v>
+      </c>
+      <c r="M3" s="83"/>
+      <c r="N3" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="O3" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="P3" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="Q3" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="R3" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="S3" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="T3" s="22"/>
+    </row>
+    <row r="4" spans="1:20" s="61" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="E4" s="89" t="s">
+        <v>118</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="H4" s="5"/>
+      <c r="I4" s="5"/>
+      <c r="J4" s="5"/>
+      <c r="K4" s="5"/>
+      <c r="L4" s="11" t="s">
+        <v>42</v>
+      </c>
+      <c r="M4" s="91" t="s">
+        <v>98</v>
+      </c>
+      <c r="N4" s="5"/>
+      <c r="O4" s="5"/>
+      <c r="P4" s="5"/>
+      <c r="Q4" s="5"/>
+      <c r="R4" s="5"/>
+      <c r="S4" s="5"/>
+      <c r="T4" s="5" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="5" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="E5" s="89" t="s">
+        <v>31</v>
+      </c>
+      <c r="G5" s="9"/>
+      <c r="H5" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="I5" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="J5" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="K5" s="90" t="s">
+        <v>32</v>
+      </c>
+      <c r="L5" s="90" t="s">
+        <v>32</v>
+      </c>
+      <c r="M5" s="9"/>
+      <c r="N5" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="O5" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="P5" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="Q5" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="R5" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="S5" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="T5" s="11" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="6" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="E6" s="89" t="s">
+        <v>117</v>
+      </c>
+      <c r="G6" s="6" t="s">
+        <v>119</v>
+      </c>
+      <c r="H6" s="9"/>
+      <c r="I6" s="9"/>
+      <c r="J6" s="9"/>
+      <c r="K6" s="9"/>
+      <c r="L6" s="9"/>
+      <c r="M6" s="9"/>
+      <c r="N6" s="9"/>
+      <c r="O6" s="9"/>
+      <c r="P6" s="9"/>
+      <c r="Q6" s="9"/>
+      <c r="R6" s="21" t="s">
+        <v>41</v>
+      </c>
+      <c r="S6" s="9"/>
+      <c r="T6" s="9"/>
+    </row>
+    <row r="7" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="C7" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>116</v>
+      </c>
+      <c r="G7" s="87"/>
+      <c r="L7" s="88"/>
+      <c r="Q7" s="29"/>
+      <c r="R7" s="92"/>
+      <c r="T7" s="64"/>
+    </row>
+    <row r="8" spans="1:20" s="14" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B8" s="70" t="s">
+        <v>108</v>
+      </c>
+      <c r="C8" s="59" t="s">
+        <v>79</v>
+      </c>
+      <c r="D8" s="69" t="s">
+        <v>105</v>
+      </c>
+      <c r="E8" s="72" t="s">
+        <v>47</v>
+      </c>
+      <c r="F8" s="79"/>
+      <c r="G8" s="60"/>
+      <c r="H8" s="34" t="s">
+        <v>51</v>
+      </c>
+      <c r="I8" s="34" t="s">
+        <v>50</v>
+      </c>
+      <c r="J8" s="34" t="s">
+        <v>49</v>
+      </c>
+      <c r="K8" s="35" t="s">
+        <v>46</v>
+      </c>
+      <c r="L8" s="65" t="s">
+        <v>52</v>
+      </c>
+      <c r="M8" s="66"/>
+      <c r="N8" s="34" t="s">
+        <v>53</v>
+      </c>
+      <c r="O8" s="34" t="s">
+        <v>63</v>
+      </c>
+      <c r="P8" s="34" t="s">
+        <v>54</v>
+      </c>
+      <c r="Q8" s="34" t="s">
+        <v>55</v>
+      </c>
+      <c r="R8" s="34" t="s">
+        <v>56</v>
+      </c>
+      <c r="S8" s="67" t="s">
+        <v>57</v>
+      </c>
+      <c r="T8" s="68"/>
+    </row>
+    <row r="9" spans="1:20" s="14" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B9" s="56"/>
+      <c r="C9" s="59"/>
+      <c r="D9" s="69" t="s">
+        <v>106</v>
+      </c>
+      <c r="E9" s="72" t="s">
+        <v>47</v>
+      </c>
+      <c r="F9" s="79"/>
+      <c r="G9" s="60"/>
+      <c r="H9" s="34" t="s">
+        <v>51</v>
+      </c>
+      <c r="I9" s="34" t="s">
+        <v>50</v>
+      </c>
+      <c r="J9" s="34" t="s">
+        <v>49</v>
+      </c>
+      <c r="K9" s="35" t="s">
+        <v>46</v>
+      </c>
+      <c r="L9" s="65" t="s">
+        <v>52</v>
+      </c>
+      <c r="M9" s="66"/>
+      <c r="N9" s="34" t="s">
+        <v>53</v>
+      </c>
+      <c r="O9" s="34" t="s">
+        <v>63</v>
+      </c>
+      <c r="P9" s="34" t="s">
+        <v>54</v>
+      </c>
+      <c r="Q9" s="34" t="s">
+        <v>55</v>
+      </c>
+      <c r="R9" s="34" t="s">
+        <v>56</v>
+      </c>
+      <c r="S9" s="67" t="s">
+        <v>57</v>
+      </c>
+      <c r="T9" s="68"/>
+    </row>
+    <row r="10" spans="1:20" s="8" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B10" s="70" t="s">
+        <v>107</v>
+      </c>
+      <c r="C10" s="62" t="s">
+        <v>80</v>
+      </c>
+      <c r="D10" s="69" t="s">
+        <v>105</v>
+      </c>
+      <c r="E10" s="73" t="s">
+        <v>13</v>
+      </c>
+      <c r="F10" s="73"/>
+      <c r="G10" s="34" t="s">
+        <v>69</v>
+      </c>
+      <c r="H10" s="34" t="s">
+        <v>68</v>
+      </c>
+      <c r="I10" s="34" t="s">
+        <v>61</v>
+      </c>
+      <c r="J10" s="34" t="s">
+        <v>67</v>
+      </c>
+      <c r="K10" s="34" t="s">
+        <v>60</v>
+      </c>
+      <c r="L10" s="34" t="s">
+        <v>64</v>
+      </c>
+      <c r="M10" s="34" t="s">
+        <v>102</v>
+      </c>
+      <c r="N10" s="34" t="s">
+        <v>103</v>
+      </c>
+      <c r="O10" s="34" t="s">
+        <v>65</v>
+      </c>
+      <c r="P10" s="34" t="s">
+        <v>62</v>
+      </c>
+      <c r="Q10" s="34" t="s">
+        <v>71</v>
+      </c>
+      <c r="R10" s="34" t="s">
+        <v>70</v>
+      </c>
+      <c r="S10" s="65" t="s">
+        <v>72</v>
+      </c>
+      <c r="T10" s="66"/>
+    </row>
+    <row r="11" spans="1:20" s="8" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B11" s="56"/>
+      <c r="C11" s="63"/>
+      <c r="D11" s="69" t="s">
+        <v>106</v>
+      </c>
+      <c r="E11" s="73" t="s">
+        <v>14</v>
+      </c>
+      <c r="F11" s="73"/>
+      <c r="G11" s="34" t="s">
+        <v>87</v>
+      </c>
+      <c r="H11" s="34" t="s">
+        <v>86</v>
+      </c>
+      <c r="I11" s="34" t="s">
+        <v>87</v>
+      </c>
+      <c r="J11" s="34" t="s">
+        <v>88</v>
+      </c>
+      <c r="K11" s="34" t="s">
+        <v>89</v>
+      </c>
+      <c r="L11" s="34" t="s">
+        <v>90</v>
+      </c>
+      <c r="M11" s="34" t="s">
+        <v>103</v>
+      </c>
+      <c r="N11" s="34" t="s">
+        <v>91</v>
+      </c>
+      <c r="O11" s="34" t="s">
+        <v>92</v>
+      </c>
+      <c r="P11" s="34" t="s">
+        <v>97</v>
+      </c>
+      <c r="Q11" s="34" t="s">
+        <v>93</v>
+      </c>
+      <c r="R11" s="34" t="s">
+        <v>94</v>
+      </c>
+      <c r="S11" s="65" t="s">
+        <v>95</v>
+      </c>
+      <c r="T11" s="66"/>
+    </row>
+    <row r="12" spans="1:20" s="8" customFormat="1" ht="26" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B12" s="71" t="s">
+        <v>75</v>
+      </c>
+      <c r="C12" s="59" t="s">
+        <v>81</v>
+      </c>
+      <c r="D12" s="69" t="s">
+        <v>105</v>
+      </c>
+      <c r="E12" s="74" t="s">
+        <v>16</v>
+      </c>
+      <c r="F12" s="80"/>
+      <c r="Q12" s="34" t="s">
+        <v>82</v>
+      </c>
+      <c r="R12" s="27" t="s">
+        <v>44</v>
+      </c>
+      <c r="S12" s="34" t="s">
+        <v>73</v>
+      </c>
+      <c r="T12" s="34" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="13" spans="1:20" s="8" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="B13" s="71"/>
+      <c r="C13" s="59"/>
+      <c r="D13" s="69" t="s">
+        <v>106</v>
+      </c>
+      <c r="E13" s="74" t="s">
+        <v>15</v>
+      </c>
+      <c r="F13" s="80"/>
+      <c r="Q13" s="34" t="s">
+        <v>83</v>
+      </c>
+      <c r="R13" s="27" t="s">
+        <v>44</v>
+      </c>
+      <c r="S13" s="34" t="s">
+        <v>76</v>
+      </c>
+      <c r="T13" s="34" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="15" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="C15" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="D15" s="5" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="16" spans="1:20" ht="33" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B16" s="71" t="s">
+        <v>113</v>
+      </c>
+      <c r="C16" s="81" t="s">
+        <v>0</v>
+      </c>
+      <c r="D16" s="25" t="s">
+        <v>17</v>
+      </c>
+      <c r="E16" s="10"/>
+      <c r="F16" s="10"/>
+      <c r="G16" s="85" t="s">
+        <v>112</v>
+      </c>
+      <c r="H16" s="85" t="s">
+        <v>112</v>
+      </c>
+      <c r="I16" s="85" t="s">
+        <v>112</v>
+      </c>
+      <c r="J16" s="85" t="s">
+        <v>112</v>
+      </c>
+      <c r="K16" s="85" t="s">
+        <v>112</v>
+      </c>
+      <c r="L16" s="85" t="s">
+        <v>112</v>
+      </c>
+      <c r="M16" s="85" t="s">
+        <v>112</v>
+      </c>
+      <c r="N16" s="85" t="s">
+        <v>112</v>
+      </c>
+      <c r="O16" s="85" t="s">
+        <v>112</v>
+      </c>
+      <c r="P16" s="85" t="s">
+        <v>112</v>
+      </c>
+      <c r="Q16" s="85" t="s">
+        <v>112</v>
+      </c>
+      <c r="R16" s="85" t="s">
+        <v>112</v>
+      </c>
+      <c r="S16" s="86" t="s">
+        <v>112</v>
+      </c>
+      <c r="T16" s="78"/>
+    </row>
+    <row r="17" spans="2:20" ht="33" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B17" s="71"/>
+      <c r="C17" s="82" t="s">
+        <v>19</v>
+      </c>
+      <c r="D17" s="23" t="s">
+        <v>18</v>
+      </c>
+      <c r="G17" s="22"/>
+      <c r="H17" s="22"/>
+      <c r="I17" s="22"/>
+      <c r="J17" s="22"/>
+      <c r="K17" s="22"/>
+      <c r="L17" s="22"/>
+      <c r="M17" s="22"/>
+      <c r="N17" s="22"/>
+      <c r="O17" s="22"/>
+      <c r="P17" s="22" t="s">
+        <v>58</v>
+      </c>
+      <c r="Q17" s="39" t="s">
+        <v>110</v>
+      </c>
+      <c r="R17" s="27" t="s">
+        <v>44</v>
+      </c>
+      <c r="S17" s="22"/>
+      <c r="T17" s="22"/>
+    </row>
+    <row r="18" spans="2:20" ht="33" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B18" s="71"/>
+      <c r="C18" s="82"/>
+      <c r="D18" s="25" t="s">
+        <v>17</v>
+      </c>
+      <c r="G18" s="22"/>
+      <c r="H18" s="22"/>
+      <c r="I18" s="22"/>
+      <c r="J18" s="22"/>
+      <c r="K18" s="22"/>
+      <c r="L18" s="38" t="s">
+        <v>101</v>
+      </c>
+      <c r="M18" s="38" t="s">
+        <v>101</v>
+      </c>
+      <c r="N18" s="22"/>
+      <c r="O18" s="22"/>
+      <c r="P18" s="38" t="s">
+        <v>111</v>
+      </c>
+      <c r="Q18" s="38" t="s">
+        <v>111</v>
+      </c>
+      <c r="R18" s="38" t="s">
+        <v>111</v>
+      </c>
+      <c r="S18" s="22"/>
+      <c r="T18" s="22"/>
+    </row>
+    <row r="19" spans="2:20" ht="33" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B19" s="71"/>
+      <c r="C19" s="82" t="s">
+        <v>20</v>
+      </c>
+      <c r="D19" s="23" t="s">
+        <v>18</v>
+      </c>
+      <c r="G19" s="22"/>
+      <c r="H19" s="22"/>
+      <c r="I19" s="22"/>
+      <c r="J19" s="22"/>
+      <c r="K19" s="22"/>
+      <c r="L19" s="22"/>
+      <c r="M19" s="22"/>
+      <c r="N19" s="22"/>
+      <c r="O19" s="22"/>
+      <c r="P19" s="22" t="s">
+        <v>58</v>
+      </c>
+      <c r="Q19" s="22"/>
+      <c r="R19" s="22"/>
+      <c r="S19" s="39" t="s">
+        <v>110</v>
+      </c>
+      <c r="T19" s="39" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="20" spans="2:20" ht="33" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B20" s="71"/>
+      <c r="C20" s="82"/>
+      <c r="D20" s="25" t="s">
+        <v>17</v>
+      </c>
+      <c r="G20" s="22"/>
+      <c r="H20" s="22"/>
+      <c r="I20" s="22"/>
+      <c r="J20" s="22"/>
+      <c r="K20" s="22"/>
+      <c r="L20" s="38" t="s">
+        <v>101</v>
+      </c>
+      <c r="M20" s="22"/>
+      <c r="N20" s="22"/>
+      <c r="O20" s="22"/>
+      <c r="P20" s="38" t="s">
+        <v>111</v>
+      </c>
+      <c r="Q20" s="22"/>
+      <c r="R20" s="22"/>
+      <c r="S20" s="84" t="s">
+        <v>111</v>
+      </c>
+      <c r="T20" s="84"/>
+    </row>
+    <row r="21" spans="2:20" ht="33" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B21" s="71"/>
+      <c r="C21" s="81" t="s">
+        <v>96</v>
+      </c>
+      <c r="D21" s="25" t="s">
+        <v>17</v>
+      </c>
+      <c r="G21" s="22"/>
+      <c r="H21" s="22"/>
+      <c r="I21" s="22"/>
+      <c r="J21" s="22"/>
+      <c r="K21" s="22"/>
+      <c r="L21" s="38" t="s">
+        <v>101</v>
+      </c>
+      <c r="M21" s="22"/>
+      <c r="N21" s="22"/>
+      <c r="O21" s="22"/>
+      <c r="P21" s="38" t="s">
+        <v>111</v>
+      </c>
+      <c r="Q21" s="22"/>
+      <c r="R21" s="22"/>
+      <c r="S21" s="22"/>
+      <c r="T21" s="22"/>
+    </row>
+    <row r="22" spans="2:20" ht="33" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B22" s="71"/>
+      <c r="C22" s="81" t="s">
+        <v>21</v>
+      </c>
+      <c r="D22" s="25" t="s">
+        <v>17</v>
+      </c>
+      <c r="G22" s="22"/>
+      <c r="H22" s="22"/>
+      <c r="I22" s="22"/>
+      <c r="J22" s="22"/>
+      <c r="K22" s="22"/>
+      <c r="L22" s="38" t="s">
+        <v>101</v>
+      </c>
+      <c r="M22" s="22"/>
+      <c r="N22" s="22"/>
+      <c r="O22" s="22"/>
+      <c r="P22" s="38" t="s">
+        <v>111</v>
+      </c>
+      <c r="Q22" s="22"/>
+      <c r="R22" s="22"/>
+      <c r="S22" s="22"/>
+      <c r="T22" s="22"/>
+    </row>
+    <row r="23" spans="2:20" ht="33" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B23" s="71"/>
+      <c r="C23" s="81" t="s">
+        <v>22</v>
+      </c>
+      <c r="D23" s="25" t="s">
+        <v>17</v>
+      </c>
+      <c r="G23" s="22"/>
+      <c r="H23" s="22"/>
+      <c r="I23" s="22"/>
+      <c r="J23" s="22"/>
+      <c r="K23" s="22"/>
+      <c r="L23" s="22"/>
+      <c r="M23" s="22"/>
+      <c r="N23" s="22"/>
+      <c r="O23" s="22"/>
+      <c r="P23" s="38" t="s">
+        <v>111</v>
+      </c>
+      <c r="Q23" s="22"/>
+      <c r="R23" s="22"/>
+      <c r="S23" s="22"/>
+      <c r="T23" s="22"/>
+    </row>
+    <row r="24" spans="2:20" ht="33" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B24" s="71"/>
+      <c r="C24" s="81" t="s">
+        <v>23</v>
+      </c>
+      <c r="D24" s="25" t="s">
+        <v>17</v>
+      </c>
+      <c r="G24" s="22"/>
+      <c r="H24" s="22"/>
+      <c r="I24" s="22"/>
+      <c r="J24" s="22"/>
+      <c r="K24" s="22"/>
+      <c r="L24" s="22"/>
+      <c r="M24" s="22"/>
+      <c r="N24" s="22"/>
+      <c r="O24" s="22"/>
+      <c r="P24" s="38" t="s">
+        <v>111</v>
+      </c>
+      <c r="Q24" s="22"/>
+      <c r="R24" s="22"/>
+      <c r="S24" s="22"/>
+      <c r="T24" s="22"/>
+    </row>
+    <row r="25" spans="2:20" ht="33" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B25" s="71"/>
+      <c r="C25" s="81" t="s">
+        <v>29</v>
+      </c>
+      <c r="D25" s="25" t="s">
+        <v>17</v>
+      </c>
+      <c r="G25" s="22"/>
+      <c r="H25" s="22"/>
+      <c r="I25" s="22"/>
+      <c r="J25" s="38" t="s">
+        <v>101</v>
+      </c>
+      <c r="K25" s="22"/>
+      <c r="L25" s="22"/>
+      <c r="M25" s="22"/>
+      <c r="N25" s="22"/>
+      <c r="O25" s="22"/>
+      <c r="P25" s="38" t="s">
+        <v>111</v>
+      </c>
+      <c r="Q25" s="22"/>
+      <c r="R25" s="22"/>
+      <c r="S25" s="22"/>
+      <c r="T25" s="22"/>
+    </row>
+    <row r="26" spans="2:20" ht="33" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B26" s="71"/>
+      <c r="C26" s="81" t="s">
+        <v>24</v>
+      </c>
+      <c r="D26" s="25" t="s">
+        <v>17</v>
+      </c>
+      <c r="G26" s="22"/>
+      <c r="H26" s="22"/>
+      <c r="I26" s="22"/>
+      <c r="J26" s="22"/>
+      <c r="K26" s="22"/>
+      <c r="L26" s="22"/>
+      <c r="M26" s="22"/>
+      <c r="N26" s="22"/>
+      <c r="O26" s="22"/>
+      <c r="P26" s="22" t="s">
+        <v>58</v>
+      </c>
+      <c r="Q26" s="22"/>
+      <c r="R26" s="22"/>
+      <c r="S26" s="22"/>
+      <c r="T26" s="22"/>
+    </row>
+    <row r="27" spans="2:20" ht="33" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B27" s="71"/>
+      <c r="C27" s="81" t="s">
+        <v>25</v>
+      </c>
+      <c r="D27" s="25" t="s">
+        <v>17</v>
+      </c>
+      <c r="G27" s="22"/>
+      <c r="H27" s="22"/>
+      <c r="I27" s="22"/>
+      <c r="J27" s="22"/>
+      <c r="K27" s="22"/>
+      <c r="L27" s="38" t="s">
+        <v>101</v>
+      </c>
+      <c r="M27" s="22"/>
+      <c r="N27" s="22"/>
+      <c r="O27" s="22"/>
+      <c r="P27" s="22" t="s">
+        <v>58</v>
+      </c>
+      <c r="Q27" s="22"/>
+      <c r="R27" s="22"/>
+      <c r="S27" s="22"/>
+      <c r="T27" s="22"/>
+    </row>
+  </sheetData>
+  <mergeCells count="18">
+    <mergeCell ref="B12:B13"/>
+    <mergeCell ref="C12:C13"/>
+    <mergeCell ref="S16:T16"/>
+    <mergeCell ref="C17:C18"/>
+    <mergeCell ref="C19:C20"/>
+    <mergeCell ref="B16:B27"/>
+    <mergeCell ref="S20:T20"/>
+    <mergeCell ref="S10:T10"/>
+    <mergeCell ref="S11:T11"/>
+    <mergeCell ref="L3:M3"/>
+    <mergeCell ref="L8:M8"/>
+    <mergeCell ref="L9:M9"/>
+    <mergeCell ref="S8:T8"/>
+    <mergeCell ref="S9:T9"/>
+    <mergeCell ref="C8:C9"/>
+    <mergeCell ref="B8:B9"/>
+    <mergeCell ref="B10:B11"/>
+    <mergeCell ref="C10:C11"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
add a display nothing config option to the config selector
</commit_message>
<xml_diff>
--- a/app/docs/Spreadhsheets/Scope Structure.xlsx
+++ b/app/docs/Spreadhsheets/Scope Structure.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/robhay/Developer/share_screener/app/docs/Spreadhsheets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5ABD55C9-F674-F045-AEC4-664C7DBDDE3D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E3CF2DE-3F04-EA4D-8A4E-CDC747D55550}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="21580" activeTab="1" xr2:uid="{952C95C7-3405-C54E-B78D-3397068AE8B3}"/>
+    <workbookView xWindow="73120" yWindow="-3700" windowWidth="38080" windowHeight="20800" activeTab="1" xr2:uid="{952C95C7-3405-C54E-B78D-3397068AE8B3}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="503" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="510" uniqueCount="125">
   <si>
     <t>Scope</t>
   </si>
@@ -392,6 +392,21 @@
   </si>
   <si>
     <t>overview of all scope</t>
+  </si>
+  <si>
+    <t>show_config_summary</t>
+  </si>
+  <si>
+    <t>display</t>
+  </si>
+  <si>
+    <t>scope_display</t>
+  </si>
+  <si>
+    <t>config_display</t>
+  </si>
+  <si>
+    <t>show_config_display</t>
   </si>
 </sst>
 </file>
@@ -898,9 +913,6 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -995,6 +1007,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2491,50 +2506,52 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14994931-7C6C-9340-B5B5-F2DD8D95EA73}">
-  <dimension ref="A1:AF27"/>
+  <dimension ref="A1:AG27"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="4.1640625" style="10" customWidth="1"/>
     <col min="2" max="2" width="15.6640625" style="10" customWidth="1"/>
     <col min="3" max="3" width="27.6640625" style="10" customWidth="1"/>
     <col min="4" max="4" width="9.1640625" style="10" customWidth="1"/>
-    <col min="5" max="5" width="19.6640625" style="75" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="6" style="75" customWidth="1"/>
+    <col min="5" max="5" width="19.6640625" style="74" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="6" style="74" customWidth="1"/>
     <col min="7" max="7" width="18.33203125" style="10" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="16" style="10" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="17.6640625" style="10" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="22.6640625" style="10" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="17" style="10" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="18" style="10" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="19" style="10" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="25.5" style="10" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="14" style="10" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="17.5" style="10" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="18.33203125" style="10" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="19.33203125" style="10" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="19.1640625" style="10" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="20" style="10" bestFit="1" customWidth="1"/>
-    <col min="21" max="16384" width="10.83203125" style="10"/>
+    <col min="10" max="10" width="17.6640625" style="10" customWidth="1"/>
+    <col min="11" max="11" width="22.6640625" style="10" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="17" style="10" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="18" style="10" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="19" style="10" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="25.5" style="10" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="14" style="10" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="17.5" style="10" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="18.33203125" style="10" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="19.33203125" style="10" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="19.1640625" style="10" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="20" style="10" bestFit="1" customWidth="1"/>
+    <col min="22" max="16384" width="10.83203125" style="10"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" ht="26" x14ac:dyDescent="0.2">
-      <c r="A1" s="76" t="s">
+    <row r="1" spans="1:21" ht="26" x14ac:dyDescent="0.2">
+      <c r="A1" s="75" t="s">
         <v>40</v>
       </c>
-      <c r="B1" s="76"/>
-      <c r="C1" s="76"/>
-      <c r="D1" s="76"/>
-      <c r="E1" s="77"/>
-      <c r="F1" s="77"/>
-      <c r="G1" s="76"/>
-      <c r="H1" s="76"/>
-      <c r="I1" s="76"/>
-      <c r="J1" s="76"/>
-      <c r="S1" s="76"/>
-      <c r="T1" s="76"/>
-    </row>
-    <row r="3" spans="1:20" s="61" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="E3" s="89" t="s">
+      <c r="B1" s="75"/>
+      <c r="C1" s="75"/>
+      <c r="D1" s="75"/>
+      <c r="E1" s="76"/>
+      <c r="F1" s="76"/>
+      <c r="G1" s="75"/>
+      <c r="H1" s="75"/>
+      <c r="I1" s="75"/>
+      <c r="J1" s="75"/>
+      <c r="K1" s="75"/>
+      <c r="T1" s="75"/>
+      <c r="U1" s="75"/>
+    </row>
+    <row r="3" spans="1:21" s="60" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="E3" s="88" t="s">
         <v>114</v>
       </c>
       <c r="G3" s="22"/>
@@ -2545,37 +2562,40 @@
         <v>4</v>
       </c>
       <c r="J3" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="K3" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="K3" s="5" t="s">
+      <c r="L3" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="L3" s="83" t="s">
+      <c r="M3" s="82" t="s">
         <v>7</v>
       </c>
-      <c r="M3" s="83"/>
-      <c r="N3" s="5" t="s">
+      <c r="N3" s="82"/>
+      <c r="O3" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="O3" s="5" t="s">
+      <c r="P3" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="P3" s="5" t="s">
+      <c r="Q3" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="Q3" s="5" t="s">
+      <c r="R3" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="R3" s="5" t="s">
+      <c r="S3" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="S3" s="5" t="s">
+      <c r="T3" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="T3" s="22"/>
-    </row>
-    <row r="4" spans="1:20" s="61" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="E4" s="89" t="s">
+      <c r="U3" s="22"/>
+    </row>
+    <row r="4" spans="1:21" s="60" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="E4" s="88" t="s">
         <v>118</v>
       </c>
       <c r="G4" s="5" t="s">
@@ -2585,24 +2605,25 @@
       <c r="I4" s="5"/>
       <c r="J4" s="5"/>
       <c r="K4" s="5"/>
-      <c r="L4" s="11" t="s">
+      <c r="L4" s="5"/>
+      <c r="M4" s="11" t="s">
         <v>42</v>
       </c>
-      <c r="M4" s="91" t="s">
+      <c r="N4" s="90" t="s">
         <v>98</v>
       </c>
-      <c r="N4" s="5"/>
       <c r="O4" s="5"/>
       <c r="P4" s="5"/>
       <c r="Q4" s="5"/>
       <c r="R4" s="5"/>
       <c r="S4" s="5"/>
-      <c r="T4" s="5" t="s">
+      <c r="T4" s="5"/>
+      <c r="U4" s="5" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="E5" s="89" t="s">
+    <row r="5" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="E5" s="88" t="s">
         <v>31</v>
       </c>
       <c r="G5" s="9"/>
@@ -2615,16 +2636,16 @@
       <c r="J5" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="K5" s="90" t="s">
+      <c r="K5" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="L5" s="89" t="s">
         <v>32</v>
       </c>
-      <c r="L5" s="90" t="s">
+      <c r="M5" s="89" t="s">
         <v>32</v>
       </c>
-      <c r="M5" s="9"/>
-      <c r="N5" s="11" t="s">
-        <v>34</v>
-      </c>
+      <c r="N5" s="9"/>
       <c r="O5" s="11" t="s">
         <v>34</v>
       </c>
@@ -2643,9 +2664,12 @@
       <c r="T5" s="11" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="E6" s="89" t="s">
+      <c r="U5" s="11" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="6" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="E6" s="88" t="s">
         <v>117</v>
       </c>
       <c r="G6" s="6" t="s">
@@ -2661,13 +2685,14 @@
       <c r="O6" s="9"/>
       <c r="P6" s="9"/>
       <c r="Q6" s="9"/>
-      <c r="R6" s="21" t="s">
+      <c r="R6" s="9"/>
+      <c r="S6" s="21" t="s">
         <v>41</v>
       </c>
-      <c r="S6" s="9"/>
       <c r="T6" s="9"/>
-    </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="U6" s="9"/>
+    </row>
+    <row r="7" spans="1:21" x14ac:dyDescent="0.2">
       <c r="C7" s="5" t="s">
         <v>115</v>
       </c>
@@ -2677,27 +2702,27 @@
       <c r="E7" s="5" t="s">
         <v>116</v>
       </c>
-      <c r="G7" s="87"/>
-      <c r="L7" s="88"/>
-      <c r="Q7" s="29"/>
-      <c r="R7" s="92"/>
-      <c r="T7" s="64"/>
-    </row>
-    <row r="8" spans="1:20" s="14" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B8" s="70" t="s">
+      <c r="G7" s="86"/>
+      <c r="M7" s="87"/>
+      <c r="R7" s="29"/>
+      <c r="S7" s="91"/>
+      <c r="U7" s="63"/>
+    </row>
+    <row r="8" spans="1:21" s="14" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B8" s="69" t="s">
         <v>108</v>
       </c>
       <c r="C8" s="59" t="s">
         <v>79</v>
       </c>
-      <c r="D8" s="69" t="s">
+      <c r="D8" s="68" t="s">
         <v>105</v>
       </c>
-      <c r="E8" s="72" t="s">
+      <c r="E8" s="71" t="s">
         <v>47</v>
       </c>
-      <c r="F8" s="79"/>
-      <c r="G8" s="60"/>
+      <c r="F8" s="78"/>
+      <c r="G8" s="22"/>
       <c r="H8" s="34" t="s">
         <v>51</v>
       </c>
@@ -2705,46 +2730,49 @@
         <v>50</v>
       </c>
       <c r="J8" s="34" t="s">
+        <v>122</v>
+      </c>
+      <c r="K8" s="34" t="s">
         <v>49</v>
       </c>
-      <c r="K8" s="35" t="s">
+      <c r="L8" s="35" t="s">
         <v>46</v>
       </c>
-      <c r="L8" s="65" t="s">
+      <c r="M8" s="64" t="s">
         <v>52</v>
       </c>
-      <c r="M8" s="66"/>
-      <c r="N8" s="34" t="s">
+      <c r="N8" s="65"/>
+      <c r="O8" s="34" t="s">
         <v>53</v>
       </c>
-      <c r="O8" s="34" t="s">
+      <c r="P8" s="34" t="s">
         <v>63</v>
       </c>
-      <c r="P8" s="34" t="s">
+      <c r="Q8" s="34" t="s">
         <v>54</v>
       </c>
-      <c r="Q8" s="34" t="s">
+      <c r="R8" s="34" t="s">
         <v>55</v>
       </c>
-      <c r="R8" s="34" t="s">
+      <c r="S8" s="34" t="s">
         <v>56</v>
       </c>
-      <c r="S8" s="67" t="s">
+      <c r="T8" s="66" t="s">
         <v>57</v>
       </c>
-      <c r="T8" s="68"/>
-    </row>
-    <row r="9" spans="1:20" s="14" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="U8" s="67"/>
+    </row>
+    <row r="9" spans="1:21" s="14" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B9" s="56"/>
       <c r="C9" s="59"/>
-      <c r="D9" s="69" t="s">
+      <c r="D9" s="68" t="s">
         <v>106</v>
       </c>
-      <c r="E9" s="72" t="s">
+      <c r="E9" s="71" t="s">
         <v>47</v>
       </c>
-      <c r="F9" s="79"/>
-      <c r="G9" s="60"/>
+      <c r="F9" s="78"/>
+      <c r="G9" s="22"/>
       <c r="H9" s="34" t="s">
         <v>51</v>
       </c>
@@ -2752,49 +2780,52 @@
         <v>50</v>
       </c>
       <c r="J9" s="34" t="s">
+        <v>122</v>
+      </c>
+      <c r="K9" s="34" t="s">
         <v>49</v>
       </c>
-      <c r="K9" s="35" t="s">
+      <c r="L9" s="35" t="s">
         <v>46</v>
       </c>
-      <c r="L9" s="65" t="s">
+      <c r="M9" s="64" t="s">
         <v>52</v>
       </c>
-      <c r="M9" s="66"/>
-      <c r="N9" s="34" t="s">
+      <c r="N9" s="65"/>
+      <c r="O9" s="34" t="s">
         <v>53</v>
       </c>
-      <c r="O9" s="34" t="s">
+      <c r="P9" s="34" t="s">
         <v>63</v>
       </c>
-      <c r="P9" s="34" t="s">
+      <c r="Q9" s="34" t="s">
         <v>54</v>
       </c>
-      <c r="Q9" s="34" t="s">
+      <c r="R9" s="34" t="s">
         <v>55</v>
       </c>
-      <c r="R9" s="34" t="s">
+      <c r="S9" s="34" t="s">
         <v>56</v>
       </c>
-      <c r="S9" s="67" t="s">
+      <c r="T9" s="66" t="s">
         <v>57</v>
       </c>
-      <c r="T9" s="68"/>
-    </row>
-    <row r="10" spans="1:20" s="8" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B10" s="70" t="s">
+      <c r="U9" s="67"/>
+    </row>
+    <row r="10" spans="1:21" s="8" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B10" s="69" t="s">
         <v>107</v>
       </c>
-      <c r="C10" s="62" t="s">
+      <c r="C10" s="61" t="s">
         <v>80</v>
       </c>
-      <c r="D10" s="69" t="s">
+      <c r="D10" s="68" t="s">
         <v>105</v>
       </c>
-      <c r="E10" s="73" t="s">
+      <c r="E10" s="72" t="s">
         <v>13</v>
       </c>
-      <c r="F10" s="73"/>
+      <c r="F10" s="72"/>
       <c r="G10" s="34" t="s">
         <v>69</v>
       </c>
@@ -2805,49 +2836,52 @@
         <v>61</v>
       </c>
       <c r="J10" s="34" t="s">
+        <v>123</v>
+      </c>
+      <c r="K10" s="34" t="s">
         <v>67</v>
       </c>
-      <c r="K10" s="34" t="s">
+      <c r="L10" s="34" t="s">
         <v>60</v>
       </c>
-      <c r="L10" s="34" t="s">
+      <c r="M10" s="34" t="s">
         <v>64</v>
       </c>
-      <c r="M10" s="34" t="s">
+      <c r="N10" s="34" t="s">
         <v>102</v>
       </c>
-      <c r="N10" s="34" t="s">
+      <c r="O10" s="34" t="s">
         <v>103</v>
       </c>
-      <c r="O10" s="34" t="s">
+      <c r="P10" s="34" t="s">
         <v>65</v>
       </c>
-      <c r="P10" s="34" t="s">
+      <c r="Q10" s="34" t="s">
         <v>62</v>
       </c>
-      <c r="Q10" s="34" t="s">
+      <c r="R10" s="34" t="s">
         <v>71</v>
       </c>
-      <c r="R10" s="34" t="s">
+      <c r="S10" s="34" t="s">
         <v>70</v>
       </c>
-      <c r="S10" s="65" t="s">
+      <c r="T10" s="64" t="s">
         <v>72</v>
       </c>
-      <c r="T10" s="66"/>
-    </row>
-    <row r="11" spans="1:20" s="8" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="U10" s="65"/>
+    </row>
+    <row r="11" spans="1:21" s="8" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B11" s="56"/>
-      <c r="C11" s="63"/>
-      <c r="D11" s="69" t="s">
+      <c r="C11" s="62"/>
+      <c r="D11" s="68" t="s">
         <v>106</v>
       </c>
-      <c r="E11" s="73" t="s">
+      <c r="E11" s="72" t="s">
         <v>14</v>
       </c>
-      <c r="F11" s="73"/>
+      <c r="F11" s="72"/>
       <c r="G11" s="34" t="s">
-        <v>87</v>
+        <v>120</v>
       </c>
       <c r="H11" s="34" t="s">
         <v>86</v>
@@ -2856,88 +2890,91 @@
         <v>87</v>
       </c>
       <c r="J11" s="34" t="s">
+        <v>124</v>
+      </c>
+      <c r="K11" s="34" t="s">
         <v>88</v>
       </c>
-      <c r="K11" s="34" t="s">
+      <c r="L11" s="34" t="s">
         <v>89</v>
       </c>
-      <c r="L11" s="34" t="s">
+      <c r="M11" s="34" t="s">
         <v>90</v>
       </c>
-      <c r="M11" s="34" t="s">
+      <c r="N11" s="34" t="s">
         <v>103</v>
       </c>
-      <c r="N11" s="34" t="s">
+      <c r="O11" s="34" t="s">
         <v>91</v>
       </c>
-      <c r="O11" s="34" t="s">
+      <c r="P11" s="34" t="s">
         <v>92</v>
       </c>
-      <c r="P11" s="34" t="s">
+      <c r="Q11" s="34" t="s">
         <v>97</v>
       </c>
-      <c r="Q11" s="34" t="s">
+      <c r="R11" s="34" t="s">
         <v>93</v>
       </c>
-      <c r="R11" s="34" t="s">
+      <c r="S11" s="34" t="s">
         <v>94</v>
       </c>
-      <c r="S11" s="65" t="s">
+      <c r="T11" s="64" t="s">
         <v>95</v>
       </c>
-      <c r="T11" s="66"/>
-    </row>
-    <row r="12" spans="1:20" s="8" customFormat="1" ht="26" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B12" s="71" t="s">
+      <c r="U11" s="65"/>
+    </row>
+    <row r="12" spans="1:21" s="8" customFormat="1" ht="26" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B12" s="70" t="s">
         <v>75</v>
       </c>
       <c r="C12" s="59" t="s">
         <v>81</v>
       </c>
-      <c r="D12" s="69" t="s">
+      <c r="D12" s="68" t="s">
         <v>105</v>
       </c>
-      <c r="E12" s="74" t="s">
+      <c r="E12" s="73" t="s">
         <v>16</v>
       </c>
-      <c r="F12" s="80"/>
-      <c r="Q12" s="34" t="s">
+      <c r="F12" s="79"/>
+      <c r="R12" s="34" t="s">
         <v>82</v>
       </c>
-      <c r="R12" s="27" t="s">
+      <c r="S12" s="27" t="s">
         <v>44</v>
       </c>
-      <c r="S12" s="34" t="s">
+      <c r="T12" s="34" t="s">
         <v>73</v>
       </c>
-      <c r="T12" s="34" t="s">
+      <c r="U12" s="34" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="13" spans="1:20" s="8" customFormat="1" ht="17" x14ac:dyDescent="0.2">
-      <c r="B13" s="71"/>
+    <row r="13" spans="1:21" s="8" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="B13" s="70"/>
       <c r="C13" s="59"/>
-      <c r="D13" s="69" t="s">
+      <c r="D13" s="68" t="s">
         <v>106</v>
       </c>
-      <c r="E13" s="74" t="s">
+      <c r="E13" s="73" t="s">
         <v>15</v>
       </c>
-      <c r="F13" s="80"/>
-      <c r="Q13" s="34" t="s">
+      <c r="F13" s="79"/>
+      <c r="R13" s="34" t="s">
         <v>83</v>
       </c>
-      <c r="R13" s="27" t="s">
+      <c r="S13" s="27" t="s">
         <v>44</v>
       </c>
-      <c r="S13" s="34" t="s">
+      <c r="T13" s="34" t="s">
         <v>76</v>
       </c>
-      <c r="T13" s="34" t="s">
+      <c r="U13" s="34" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="15" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:21" x14ac:dyDescent="0.2">
       <c r="C15" s="5" t="s">
         <v>109</v>
       </c>
@@ -2945,11 +2982,11 @@
         <v>31</v>
       </c>
     </row>
-    <row r="16" spans="1:20" ht="33" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B16" s="71" t="s">
+    <row r="16" spans="1:21" ht="33" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B16" s="70" t="s">
         <v>113</v>
       </c>
-      <c r="C16" s="81" t="s">
+      <c r="C16" s="80" t="s">
         <v>0</v>
       </c>
       <c r="D16" s="25" t="s">
@@ -2957,50 +2994,53 @@
       </c>
       <c r="E16" s="10"/>
       <c r="F16" s="10"/>
-      <c r="G16" s="85" t="s">
+      <c r="G16" s="84" t="s">
         <v>112</v>
       </c>
-      <c r="H16" s="85" t="s">
+      <c r="H16" s="84" t="s">
         <v>112</v>
       </c>
-      <c r="I16" s="85" t="s">
+      <c r="I16" s="84" t="s">
         <v>112</v>
       </c>
-      <c r="J16" s="85" t="s">
+      <c r="J16" s="84" t="s">
         <v>112</v>
       </c>
-      <c r="K16" s="85" t="s">
+      <c r="K16" s="84" t="s">
         <v>112</v>
       </c>
-      <c r="L16" s="85" t="s">
+      <c r="L16" s="84" t="s">
         <v>112</v>
       </c>
-      <c r="M16" s="85" t="s">
+      <c r="M16" s="84" t="s">
         <v>112</v>
       </c>
-      <c r="N16" s="85" t="s">
+      <c r="N16" s="84" t="s">
         <v>112</v>
       </c>
-      <c r="O16" s="85" t="s">
+      <c r="O16" s="84" t="s">
         <v>112</v>
       </c>
-      <c r="P16" s="85" t="s">
+      <c r="P16" s="84" t="s">
         <v>112</v>
       </c>
-      <c r="Q16" s="85" t="s">
+      <c r="Q16" s="84" t="s">
         <v>112</v>
       </c>
-      <c r="R16" s="85" t="s">
+      <c r="R16" s="84" t="s">
         <v>112</v>
       </c>
-      <c r="S16" s="86" t="s">
+      <c r="S16" s="84" t="s">
         <v>112</v>
       </c>
-      <c r="T16" s="78"/>
-    </row>
-    <row r="17" spans="2:20" ht="33" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B17" s="71"/>
-      <c r="C17" s="82" t="s">
+      <c r="T16" s="85" t="s">
+        <v>112</v>
+      </c>
+      <c r="U16" s="77"/>
+    </row>
+    <row r="17" spans="2:21" ht="33" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B17" s="70"/>
+      <c r="C17" s="81" t="s">
         <v>19</v>
       </c>
       <c r="D17" s="23" t="s">
@@ -3015,21 +3055,22 @@
       <c r="M17" s="22"/>
       <c r="N17" s="22"/>
       <c r="O17" s="22"/>
-      <c r="P17" s="22" t="s">
+      <c r="P17" s="22"/>
+      <c r="Q17" s="22" t="s">
         <v>58</v>
       </c>
-      <c r="Q17" s="39" t="s">
+      <c r="R17" s="39" t="s">
         <v>110</v>
       </c>
-      <c r="R17" s="27" t="s">
+      <c r="S17" s="27" t="s">
         <v>44</v>
       </c>
-      <c r="S17" s="22"/>
       <c r="T17" s="22"/>
-    </row>
-    <row r="18" spans="2:20" ht="33" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B18" s="71"/>
-      <c r="C18" s="82"/>
+      <c r="U17" s="22"/>
+    </row>
+    <row r="18" spans="2:21" ht="33" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B18" s="70"/>
+      <c r="C18" s="81"/>
       <c r="D18" s="25" t="s">
         <v>17</v>
       </c>
@@ -3038,29 +3079,30 @@
       <c r="I18" s="22"/>
       <c r="J18" s="22"/>
       <c r="K18" s="22"/>
-      <c r="L18" s="38" t="s">
-        <v>101</v>
-      </c>
+      <c r="L18" s="22"/>
       <c r="M18" s="38" t="s">
         <v>101</v>
       </c>
-      <c r="N18" s="22"/>
+      <c r="N18" s="38" t="s">
+        <v>101</v>
+      </c>
       <c r="O18" s="22"/>
-      <c r="P18" s="38" t="s">
-        <v>111</v>
-      </c>
+      <c r="P18" s="22"/>
       <c r="Q18" s="38" t="s">
         <v>111</v>
       </c>
       <c r="R18" s="38" t="s">
         <v>111</v>
       </c>
-      <c r="S18" s="22"/>
+      <c r="S18" s="38" t="s">
+        <v>111</v>
+      </c>
       <c r="T18" s="22"/>
-    </row>
-    <row r="19" spans="2:20" ht="33" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B19" s="71"/>
-      <c r="C19" s="82" t="s">
+      <c r="U18" s="22"/>
+    </row>
+    <row r="19" spans="2:21" ht="33" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B19" s="70"/>
+      <c r="C19" s="81" t="s">
         <v>20</v>
       </c>
       <c r="D19" s="23" t="s">
@@ -3075,21 +3117,22 @@
       <c r="M19" s="22"/>
       <c r="N19" s="22"/>
       <c r="O19" s="22"/>
-      <c r="P19" s="22" t="s">
+      <c r="P19" s="22"/>
+      <c r="Q19" s="22" t="s">
         <v>58</v>
       </c>
-      <c r="Q19" s="22"/>
       <c r="R19" s="22"/>
-      <c r="S19" s="39" t="s">
-        <v>110</v>
-      </c>
+      <c r="S19" s="22"/>
       <c r="T19" s="39" t="s">
         <v>110</v>
       </c>
-    </row>
-    <row r="20" spans="2:20" ht="33" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B20" s="71"/>
-      <c r="C20" s="82"/>
+      <c r="U19" s="39" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="20" spans="2:21" ht="33" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B20" s="70"/>
+      <c r="C20" s="81"/>
       <c r="D20" s="25" t="s">
         <v>17</v>
       </c>
@@ -3098,25 +3141,26 @@
       <c r="I20" s="22"/>
       <c r="J20" s="22"/>
       <c r="K20" s="22"/>
-      <c r="L20" s="38" t="s">
+      <c r="L20" s="22"/>
+      <c r="M20" s="38" t="s">
         <v>101</v>
       </c>
-      <c r="M20" s="22"/>
       <c r="N20" s="22"/>
       <c r="O20" s="22"/>
-      <c r="P20" s="38" t="s">
+      <c r="P20" s="22"/>
+      <c r="Q20" s="38" t="s">
         <v>111</v>
       </c>
-      <c r="Q20" s="22"/>
       <c r="R20" s="22"/>
-      <c r="S20" s="84" t="s">
+      <c r="S20" s="22"/>
+      <c r="T20" s="83" t="s">
         <v>111</v>
       </c>
-      <c r="T20" s="84"/>
-    </row>
-    <row r="21" spans="2:20" ht="33" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B21" s="71"/>
-      <c r="C21" s="81" t="s">
+      <c r="U20" s="83"/>
+    </row>
+    <row r="21" spans="2:21" ht="33" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B21" s="70"/>
+      <c r="C21" s="80" t="s">
         <v>96</v>
       </c>
       <c r="D21" s="25" t="s">
@@ -3127,23 +3171,24 @@
       <c r="I21" s="22"/>
       <c r="J21" s="22"/>
       <c r="K21" s="22"/>
-      <c r="L21" s="38" t="s">
+      <c r="L21" s="22"/>
+      <c r="M21" s="38" t="s">
         <v>101</v>
       </c>
-      <c r="M21" s="22"/>
       <c r="N21" s="22"/>
       <c r="O21" s="22"/>
-      <c r="P21" s="38" t="s">
+      <c r="P21" s="22"/>
+      <c r="Q21" s="38" t="s">
         <v>111</v>
       </c>
-      <c r="Q21" s="22"/>
       <c r="R21" s="22"/>
       <c r="S21" s="22"/>
       <c r="T21" s="22"/>
-    </row>
-    <row r="22" spans="2:20" ht="33" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B22" s="71"/>
-      <c r="C22" s="81" t="s">
+      <c r="U21" s="22"/>
+    </row>
+    <row r="22" spans="2:21" ht="33" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B22" s="70"/>
+      <c r="C22" s="80" t="s">
         <v>21</v>
       </c>
       <c r="D22" s="25" t="s">
@@ -3154,23 +3199,24 @@
       <c r="I22" s="22"/>
       <c r="J22" s="22"/>
       <c r="K22" s="22"/>
-      <c r="L22" s="38" t="s">
+      <c r="L22" s="22"/>
+      <c r="M22" s="38" t="s">
         <v>101</v>
       </c>
-      <c r="M22" s="22"/>
       <c r="N22" s="22"/>
       <c r="O22" s="22"/>
-      <c r="P22" s="38" t="s">
+      <c r="P22" s="22"/>
+      <c r="Q22" s="38" t="s">
         <v>111</v>
       </c>
-      <c r="Q22" s="22"/>
       <c r="R22" s="22"/>
       <c r="S22" s="22"/>
       <c r="T22" s="22"/>
-    </row>
-    <row r="23" spans="2:20" ht="33" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B23" s="71"/>
-      <c r="C23" s="81" t="s">
+      <c r="U22" s="22"/>
+    </row>
+    <row r="23" spans="2:21" ht="33" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B23" s="70"/>
+      <c r="C23" s="80" t="s">
         <v>22</v>
       </c>
       <c r="D23" s="25" t="s">
@@ -3185,17 +3231,18 @@
       <c r="M23" s="22"/>
       <c r="N23" s="22"/>
       <c r="O23" s="22"/>
-      <c r="P23" s="38" t="s">
+      <c r="P23" s="22"/>
+      <c r="Q23" s="38" t="s">
         <v>111</v>
       </c>
-      <c r="Q23" s="22"/>
       <c r="R23" s="22"/>
       <c r="S23" s="22"/>
       <c r="T23" s="22"/>
-    </row>
-    <row r="24" spans="2:20" ht="33" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B24" s="71"/>
-      <c r="C24" s="81" t="s">
+      <c r="U23" s="22"/>
+    </row>
+    <row r="24" spans="2:21" ht="33" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B24" s="70"/>
+      <c r="C24" s="80" t="s">
         <v>23</v>
       </c>
       <c r="D24" s="25" t="s">
@@ -3210,17 +3257,18 @@
       <c r="M24" s="22"/>
       <c r="N24" s="22"/>
       <c r="O24" s="22"/>
-      <c r="P24" s="38" t="s">
+      <c r="P24" s="22"/>
+      <c r="Q24" s="38" t="s">
         <v>111</v>
       </c>
-      <c r="Q24" s="22"/>
       <c r="R24" s="22"/>
       <c r="S24" s="22"/>
       <c r="T24" s="22"/>
-    </row>
-    <row r="25" spans="2:20" ht="33" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B25" s="71"/>
-      <c r="C25" s="81" t="s">
+      <c r="U24" s="22"/>
+    </row>
+    <row r="25" spans="2:21" ht="33" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B25" s="70"/>
+      <c r="C25" s="80" t="s">
         <v>29</v>
       </c>
       <c r="D25" s="25" t="s">
@@ -3229,25 +3277,26 @@
       <c r="G25" s="22"/>
       <c r="H25" s="22"/>
       <c r="I25" s="22"/>
-      <c r="J25" s="38" t="s">
+      <c r="J25" s="92"/>
+      <c r="K25" s="38" t="s">
         <v>101</v>
       </c>
-      <c r="K25" s="22"/>
       <c r="L25" s="22"/>
       <c r="M25" s="22"/>
       <c r="N25" s="22"/>
       <c r="O25" s="22"/>
-      <c r="P25" s="38" t="s">
+      <c r="P25" s="22"/>
+      <c r="Q25" s="38" t="s">
         <v>111</v>
       </c>
-      <c r="Q25" s="22"/>
       <c r="R25" s="22"/>
       <c r="S25" s="22"/>
       <c r="T25" s="22"/>
-    </row>
-    <row r="26" spans="2:20" ht="33" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B26" s="71"/>
-      <c r="C26" s="81" t="s">
+      <c r="U25" s="22"/>
+    </row>
+    <row r="26" spans="2:21" ht="33" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B26" s="70"/>
+      <c r="C26" s="80" t="s">
         <v>24</v>
       </c>
       <c r="D26" s="25" t="s">
@@ -3262,17 +3311,18 @@
       <c r="M26" s="22"/>
       <c r="N26" s="22"/>
       <c r="O26" s="22"/>
-      <c r="P26" s="22" t="s">
+      <c r="P26" s="22"/>
+      <c r="Q26" s="22" t="s">
         <v>58</v>
       </c>
-      <c r="Q26" s="22"/>
       <c r="R26" s="22"/>
       <c r="S26" s="22"/>
       <c r="T26" s="22"/>
-    </row>
-    <row r="27" spans="2:20" ht="33" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B27" s="71"/>
-      <c r="C27" s="81" t="s">
+      <c r="U26" s="22"/>
+    </row>
+    <row r="27" spans="2:21" ht="33" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B27" s="70"/>
+      <c r="C27" s="80" t="s">
         <v>25</v>
       </c>
       <c r="D27" s="25" t="s">
@@ -3283,36 +3333,37 @@
       <c r="I27" s="22"/>
       <c r="J27" s="22"/>
       <c r="K27" s="22"/>
-      <c r="L27" s="38" t="s">
+      <c r="L27" s="22"/>
+      <c r="M27" s="38" t="s">
         <v>101</v>
       </c>
-      <c r="M27" s="22"/>
       <c r="N27" s="22"/>
       <c r="O27" s="22"/>
-      <c r="P27" s="22" t="s">
+      <c r="P27" s="22"/>
+      <c r="Q27" s="22" t="s">
         <v>58</v>
       </c>
-      <c r="Q27" s="22"/>
       <c r="R27" s="22"/>
       <c r="S27" s="22"/>
       <c r="T27" s="22"/>
+      <c r="U27" s="22"/>
     </row>
   </sheetData>
   <mergeCells count="18">
     <mergeCell ref="B12:B13"/>
     <mergeCell ref="C12:C13"/>
-    <mergeCell ref="S16:T16"/>
+    <mergeCell ref="T16:U16"/>
     <mergeCell ref="C17:C18"/>
     <mergeCell ref="C19:C20"/>
     <mergeCell ref="B16:B27"/>
-    <mergeCell ref="S20:T20"/>
-    <mergeCell ref="S10:T10"/>
-    <mergeCell ref="S11:T11"/>
-    <mergeCell ref="L3:M3"/>
-    <mergeCell ref="L8:M8"/>
-    <mergeCell ref="L9:M9"/>
-    <mergeCell ref="S8:T8"/>
-    <mergeCell ref="S9:T9"/>
+    <mergeCell ref="T20:U20"/>
+    <mergeCell ref="T10:U10"/>
+    <mergeCell ref="T11:U11"/>
+    <mergeCell ref="M3:N3"/>
+    <mergeCell ref="M8:N8"/>
+    <mergeCell ref="M9:N9"/>
+    <mergeCell ref="T8:U8"/>
+    <mergeCell ref="T9:U9"/>
     <mergeCell ref="C8:C9"/>
     <mergeCell ref="B8:B9"/>
     <mergeCell ref="B10:B11"/>

</xml_diff>